<commit_message>
Renumber the reworked EB cases so they stop overwriting the original's spec
input/EB-tests.docx is now in the repository and owns TC-EB-001, which the
rework was also using. Generating from one document then the other silently
replaced generated/TC-EB-001.spec.js, and whichever ran last won - the exact
class of quiet overwrite this project exists to avoid.

The rework is now TC-TNEB-001..003. The hand-written document keeps TC-EB-001
and stays as it is: it is worth keeping unchanged, because the three rules in
scripts/build-tneb-inputs.js are easier to see with the before and after side
by side.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FtkxF2HWgKorSaS1yzUxWk
</commit_message>
<xml_diff>
--- a/input/tneb-tests.xlsx
+++ b/input/tneb-tests.xlsx
@@ -28,7 +28,7 @@
     <t>ExpectedResult</t>
   </si>
   <si>
-    <t>TC-EB-001</t>
+    <t>TC-TNEB-001</t>
   </si>
   <si>
     <t>Download an e-Invoice</t>
@@ -91,7 +91,7 @@
     <t>Nothing was rejected</t>
   </si>
   <si>
-    <t>TC-EB-002</t>
+    <t>TC-TNEB-002</t>
   </si>
   <si>
     <t>The e-Invoice form is reachable without signing in</t>
@@ -127,7 +127,7 @@
     <t>Both download options are offered</t>
   </si>
   <si>
-    <t>TC-EB-003</t>
+    <t>TC-TNEB-003</t>
   </si>
   <si>
     <t>Malformed details return no invoice</t>

</xml_diff>

<commit_message>
Read TNEB account details from .env and skip CarInfo specs by default
The EB and TNEB test cases now name the consumer and mobile numbers as
<consumer no> and <mobile no>; the generated specs read TNEB_CONSUMER_NO and
TNEB_MOBILE_NO from .env at run time. Placeholders may contain spaces, may be
written without quotes, and work in "contains" assertions.

CarInfo specs are still generated but ignored by Playwright unless
RUN_CARINFO=1 is set.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JbRUGT6aSs4TxFgmXfvDFn
</commit_message>
<xml_diff>
--- a/input/tneb-tests.xlsx
+++ b/input/tneb-tests.xlsx
@@ -49,13 +49,13 @@
     <t>The e-Invoice form is displayed</t>
   </si>
   <si>
-    <t>Enter "123456789012" in the Consumer No box</t>
+    <t>Enter "&lt;consumer no&gt;" in the Consumer No box</t>
   </si>
   <si>
     <t>The consumer number is entered</t>
   </si>
   <si>
-    <t>Enter "9000000000" in the Registered Mobile No box</t>
+    <t>Enter "&lt;mobile no&gt;" in the Registered Mobile No box</t>
   </si>
   <si>
     <t>The mobile number is entered</t>
@@ -79,7 +79,7 @@
     <t>The bill is shown</t>
   </si>
   <si>
-    <t>Verify that the invoice summary contains "123456789012"</t>
+    <t>Verify that the invoice summary contains "&lt;consumer no&gt;"</t>
   </si>
   <si>
     <t>The bill is for this consumer</t>

</xml_diff>